<commit_message>
fix: corrige apontamentos do professor na Elaboração (#28)
</commit_message>
<xml_diff>
--- a/6.Gerenciamento de Projeto/HH - Planejamento e Controle do Projeto.xlsx
+++ b/6.Gerenciamento de Projeto/HH - Planejamento e Controle do Projeto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabio\Desktop\Faculdade\hobbyhub\6.Gerenciamento de Projeto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B526D0-5087-4D8A-AEC4-3427224981D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ABD92F7-AED8-47A3-9671-486B88799898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{31237A52-FFD1-4E1D-B5BB-391D11929C61}"/>
   </bookViews>
@@ -5626,7 +5626,7 @@
     <t>Modelar, Implementar e UC04 - Visualizar perfil de usuários</t>
   </si>
   <si>
-    <t>Protótipo de Arquitetura + UC5(Postar)</t>
+    <t>Protótipo de Arquitetura + UC05 (Postar)</t>
   </si>
   <si>
     <t>Em execução</t>
@@ -6554,6 +6554,16 @@
     <xf numFmtId="170" fontId="39" fillId="0" borderId="8" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="39" fillId="3" borderId="1" xfId="10" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="28" fillId="3" borderId="1" xfId="10" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="14" borderId="1" xfId="10" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="25" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
@@ -6627,12 +6637,15 @@
     <xf numFmtId="164" fontId="29" fillId="15" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="28" fillId="14" borderId="4" xfId="10" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="14" borderId="9" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="28" fillId="14" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="28" fillId="14" borderId="9" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="28" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6665,19 +6678,6 @@
     </xf>
     <xf numFmtId="164" fontId="27" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="39" fillId="3" borderId="1" xfId="10" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="28" fillId="3" borderId="1" xfId="10" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="28" fillId="14" borderId="1" xfId="10" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="28" fillId="14" borderId="4" xfId="10" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="17">
@@ -8564,18 +8564,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1024" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="123" t="s">
+      <c r="A1" s="126" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="123"/>
-      <c r="C1" s="123"/>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
     </row>
     <row r="2" spans="1:1024" ht="24.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="124" t="s">
+      <c r="A2" s="127" t="s">
         <v>217</v>
       </c>
-      <c r="B2" s="124"/>
-      <c r="C2" s="124"/>
+      <c r="B2" s="127"/>
+      <c r="C2" s="127"/>
     </row>
     <row r="3" spans="1:1024" ht="15" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -8727,38 +8727,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1024" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="131" t="s">
+      <c r="A1" s="134" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="131"/>
-      <c r="C1" s="131"/>
-      <c r="D1" s="131"/>
-      <c r="F1" s="125" t="s">
+      <c r="B1" s="134"/>
+      <c r="C1" s="134"/>
+      <c r="D1" s="134"/>
+      <c r="F1" s="128" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="125"/>
-      <c r="H1" s="125"/>
-      <c r="I1" s="125"/>
-      <c r="J1" s="125"/>
-      <c r="K1" s="125"/>
-      <c r="L1" s="125"/>
+      <c r="G1" s="128"/>
+      <c r="H1" s="128"/>
+      <c r="I1" s="128"/>
+      <c r="J1" s="128"/>
+      <c r="K1" s="128"/>
+      <c r="L1" s="128"/>
     </row>
     <row r="2" spans="1:1024" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="126" t="s">
+      <c r="A2" s="129" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="126"/>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="F2" s="127" t="s">
+      <c r="B2" s="129"/>
+      <c r="C2" s="129"/>
+      <c r="D2" s="129"/>
+      <c r="F2" s="130" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="127"/>
-      <c r="H2" s="127"/>
-      <c r="I2" s="127"/>
-      <c r="J2" s="127"/>
-      <c r="K2" s="127"/>
-      <c r="L2" s="127"/>
+      <c r="G2" s="130"/>
+      <c r="H2" s="130"/>
+      <c r="I2" s="130"/>
+      <c r="J2" s="130"/>
+      <c r="K2" s="130"/>
+      <c r="L2" s="130"/>
     </row>
     <row r="3" spans="1:1024" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
@@ -8779,20 +8779,20 @@
       <c r="G3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="128" t="s">
+      <c r="H3" s="131" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="128"/>
-      <c r="J3" s="128"/>
-      <c r="K3" s="128"/>
-      <c r="L3" s="128"/>
+      <c r="I3" s="131"/>
+      <c r="J3" s="131"/>
+      <c r="K3" s="131"/>
+      <c r="L3" s="131"/>
     </row>
     <row r="4" spans="1:1024" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="129" t="s">
+      <c r="A4" s="132" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="129"/>
-      <c r="C4" s="129"/>
+      <c r="B4" s="132"/>
+      <c r="C4" s="132"/>
       <c r="D4" s="8" t="s">
         <v>17</v>
       </c>
@@ -9035,11 +9035,11 @@
       </c>
     </row>
     <row r="11" spans="1:1024" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="129" t="s">
+      <c r="A11" s="132" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="129"/>
-      <c r="C11" s="129"/>
+      <c r="B11" s="132"/>
+      <c r="C11" s="132"/>
       <c r="D11" s="8">
         <f>SUM(D5:D10)</f>
         <v>48</v>
@@ -9268,11 +9268,11 @@
       <c r="L20" s="18"/>
     </row>
     <row r="21" spans="1:1024" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="129" t="s">
+      <c r="A21" s="132" t="s">
         <v>39</v>
       </c>
-      <c r="B21" s="129"/>
-      <c r="C21" s="129"/>
+      <c r="B21" s="132"/>
+      <c r="C21" s="132"/>
       <c r="D21" s="8">
         <f>SUM(D12:D20)</f>
         <v>65</v>
@@ -9527,11 +9527,11 @@
       </c>
     </row>
     <row r="39" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="129" t="s">
+      <c r="A39" s="132" t="s">
         <v>40</v>
       </c>
-      <c r="B39" s="129"/>
-      <c r="C39" s="129"/>
+      <c r="B39" s="132"/>
+      <c r="C39" s="132"/>
       <c r="D39" s="8">
         <f>SUM(D22:D38)</f>
         <v>120</v>
@@ -9664,9 +9664,9 @@
       </c>
     </row>
     <row r="49" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="130"/>
-      <c r="B49" s="130"/>
-      <c r="C49" s="130"/>
+      <c r="A49" s="133"/>
+      <c r="B49" s="133"/>
+      <c r="C49" s="133"/>
       <c r="D49" s="8">
         <f>SUM(D40:D48)</f>
         <v>82</v>
@@ -9712,19 +9712,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="132" t="s">
+      <c r="A1" s="135" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="132"/>
-      <c r="C1" s="132"/>
+      <c r="B1" s="135"/>
+      <c r="C1" s="135"/>
     </row>
     <row r="2" spans="1:5" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="133" t="s">
+      <c r="A3" s="136" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="133"/>
-      <c r="C3" s="133"/>
+      <c r="B3" s="136"/>
+      <c r="C3" s="136"/>
     </row>
     <row r="4" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
@@ -9833,11 +9833,11 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="133" t="s">
+      <c r="A14" s="136" t="s">
         <v>65</v>
       </c>
-      <c r="B14" s="133"/>
-      <c r="C14" s="133"/>
+      <c r="B14" s="136"/>
+      <c r="C14" s="136"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="27" t="s">
@@ -9946,54 +9946,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="122" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
+      <c r="B1" s="122"/>
+      <c r="C1" s="122"/>
+      <c r="D1" s="122"/>
+      <c r="E1" s="122"/>
+      <c r="F1" s="122"/>
+      <c r="G1" s="122"/>
+      <c r="H1" s="122"/>
+      <c r="I1" s="122"/>
+      <c r="J1" s="122"/>
+      <c r="K1" s="122"/>
     </row>
     <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="120" t="s">
+      <c r="A2" s="123" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="120"/>
-      <c r="C2" s="120"/>
-      <c r="D2" s="120"/>
+      <c r="B2" s="123"/>
+      <c r="C2" s="123"/>
+      <c r="D2" s="123"/>
       <c r="E2" s="41">
         <f>Planejamento!$B$10</f>
         <v>456.75</v>
       </c>
       <c r="F2" s="42"/>
-      <c r="G2" s="120" t="s">
+      <c r="G2" s="123" t="s">
         <v>75</v>
       </c>
-      <c r="H2" s="120"/>
-      <c r="I2" s="120"/>
-      <c r="J2" s="120"/>
+      <c r="H2" s="123"/>
+      <c r="I2" s="123"/>
+      <c r="J2" s="123"/>
       <c r="K2" s="41"/>
     </row>
     <row r="3" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="43"/>
       <c r="B3" s="44"/>
-      <c r="C3" s="121" t="s">
+      <c r="C3" s="124" t="s">
         <v>76</v>
       </c>
-      <c r="D3" s="121"/>
-      <c r="E3" s="121"/>
+      <c r="D3" s="124"/>
+      <c r="E3" s="124"/>
       <c r="F3" s="45"/>
-      <c r="G3" s="122" t="s">
+      <c r="G3" s="125" t="s">
         <v>77</v>
       </c>
-      <c r="H3" s="122"/>
-      <c r="I3" s="122"/>
+      <c r="H3" s="125"/>
+      <c r="I3" s="125"/>
       <c r="J3" s="47"/>
       <c r="K3" s="48"/>
     </row>
@@ -10064,7 +10064,7 @@
         <f>E5-I5</f>
         <v>10</v>
       </c>
-      <c r="K5" s="157" t="s">
+      <c r="K5" s="119" t="s">
         <v>270</v>
       </c>
     </row>
@@ -10091,7 +10091,7 @@
         <v>46280</v>
       </c>
       <c r="H6" s="109">
-        <v>46300</v>
+        <v>46315</v>
       </c>
       <c r="I6" s="112">
         <v>95</v>
@@ -10100,7 +10100,7 @@
         <f>E6-I6</f>
         <v>-10</v>
       </c>
-      <c r="K6" s="157" t="s">
+      <c r="K6" s="119" t="s">
         <v>271</v>
       </c>
     </row>
@@ -10124,12 +10124,12 @@
         <v>267</v>
       </c>
       <c r="G7" s="109">
-        <v>46297</v>
+        <v>46315</v>
       </c>
       <c r="H7" s="109"/>
       <c r="I7" s="112"/>
       <c r="J7" s="113"/>
-      <c r="K7" s="157" t="s">
+      <c r="K7" s="119" t="s">
         <v>272</v>
       </c>
     </row>
@@ -10150,13 +10150,13 @@
         <v>82</v>
       </c>
       <c r="F8" s="110" t="s">
-        <v>88</v>
+        <v>267</v>
       </c>
       <c r="G8" s="109"/>
       <c r="H8" s="109"/>
       <c r="I8" s="112"/>
       <c r="J8" s="113"/>
-      <c r="K8" s="157" t="s">
+      <c r="K8" s="119" t="s">
         <v>273</v>
       </c>
     </row>
@@ -10183,7 +10183,7 @@
       <c r="H9" s="109"/>
       <c r="I9" s="112"/>
       <c r="J9" s="113"/>
-      <c r="K9" s="157" t="s">
+      <c r="K9" s="119" t="s">
         <v>274</v>
       </c>
     </row>
@@ -10210,7 +10210,7 @@
       <c r="H10" s="109"/>
       <c r="I10" s="112"/>
       <c r="J10" s="113"/>
-      <c r="K10" s="157" t="s">
+      <c r="K10" s="119" t="s">
         <v>275</v>
       </c>
     </row>
@@ -10339,19 +10339,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="53" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="119" t="s">
+      <c r="A1" s="122" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="119"/>
-      <c r="C1" s="119"/>
-      <c r="D1" s="119"/>
-      <c r="E1" s="119"/>
-      <c r="F1" s="119"/>
-      <c r="G1" s="119"/>
-      <c r="H1" s="119"/>
-      <c r="I1" s="119"/>
-      <c r="J1" s="119"/>
-      <c r="K1" s="119"/>
+      <c r="B1" s="122"/>
+      <c r="C1" s="122"/>
+      <c r="D1" s="122"/>
+      <c r="E1" s="122"/>
+      <c r="F1" s="122"/>
+      <c r="G1" s="122"/>
+      <c r="H1" s="122"/>
+      <c r="I1" s="122"/>
+      <c r="J1" s="122"/>
+      <c r="K1" s="122"/>
     </row>
     <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -10505,10 +10505,10 @@
       </c>
     </row>
     <row r="33" spans="1:11" ht="22.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D33" s="135" t="s">
+      <c r="D33" s="138" t="s">
         <v>120</v>
       </c>
-      <c r="E33" s="135"/>
+      <c r="E33" s="138"/>
     </row>
     <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D34" s="56">
@@ -10560,137 +10560,137 @@
     </row>
     <row r="40" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:11" s="53" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="136" t="s">
+      <c r="A41" s="139" t="s">
         <v>127</v>
       </c>
-      <c r="B41" s="136"/>
-      <c r="C41" s="136"/>
-      <c r="D41" s="136"/>
-      <c r="E41" s="136"/>
-      <c r="F41" s="136"/>
-      <c r="G41" s="136"/>
-      <c r="H41" s="136"/>
-      <c r="I41" s="136"/>
-      <c r="J41" s="136"/>
-      <c r="K41" s="136"/>
+      <c r="B41" s="139"/>
+      <c r="C41" s="139"/>
+      <c r="D41" s="139"/>
+      <c r="E41" s="139"/>
+      <c r="F41" s="139"/>
+      <c r="G41" s="139"/>
+      <c r="H41" s="139"/>
+      <c r="I41" s="139"/>
+      <c r="J41" s="139"/>
+      <c r="K41" s="139"/>
     </row>
     <row r="42" spans="1:11" s="53" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="137" t="s">
+      <c r="A42" s="140" t="s">
         <v>128</v>
       </c>
-      <c r="B42" s="137"/>
-      <c r="C42" s="137"/>
-      <c r="D42" s="137"/>
-      <c r="E42" s="137"/>
-      <c r="F42" s="137"/>
-      <c r="G42" s="137"/>
-      <c r="H42" s="137"/>
-      <c r="I42" s="137"/>
-      <c r="J42" s="137"/>
-      <c r="K42" s="137"/>
+      <c r="B42" s="140"/>
+      <c r="C42" s="140"/>
+      <c r="D42" s="140"/>
+      <c r="E42" s="140"/>
+      <c r="F42" s="140"/>
+      <c r="G42" s="140"/>
+      <c r="H42" s="140"/>
+      <c r="I42" s="140"/>
+      <c r="J42" s="140"/>
+      <c r="K42" s="140"/>
     </row>
     <row r="43" spans="1:11" s="53" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="138" t="s">
+      <c r="A43" s="141" t="s">
         <v>129</v>
       </c>
-      <c r="B43" s="138"/>
-      <c r="C43" s="138"/>
-      <c r="D43" s="138"/>
-      <c r="E43" s="138"/>
-      <c r="F43" s="138"/>
-      <c r="G43" s="138"/>
-      <c r="H43" s="138"/>
-      <c r="I43" s="138"/>
-      <c r="J43" s="138"/>
-      <c r="K43" s="138"/>
+      <c r="B43" s="141"/>
+      <c r="C43" s="141"/>
+      <c r="D43" s="141"/>
+      <c r="E43" s="141"/>
+      <c r="F43" s="141"/>
+      <c r="G43" s="141"/>
+      <c r="H43" s="141"/>
+      <c r="I43" s="141"/>
+      <c r="J43" s="141"/>
+      <c r="K43" s="141"/>
     </row>
     <row r="44" spans="1:11" s="53" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="134" t="s">
+      <c r="A44" s="137" t="s">
         <v>130</v>
       </c>
-      <c r="B44" s="134"/>
-      <c r="C44" s="134"/>
-      <c r="D44" s="134"/>
-      <c r="E44" s="134"/>
-      <c r="F44" s="134"/>
-      <c r="G44" s="134"/>
-      <c r="H44" s="134"/>
-      <c r="I44" s="134"/>
-      <c r="J44" s="134"/>
-      <c r="K44" s="134"/>
+      <c r="B44" s="137"/>
+      <c r="C44" s="137"/>
+      <c r="D44" s="137"/>
+      <c r="E44" s="137"/>
+      <c r="F44" s="137"/>
+      <c r="G44" s="137"/>
+      <c r="H44" s="137"/>
+      <c r="I44" s="137"/>
+      <c r="J44" s="137"/>
+      <c r="K44" s="137"/>
     </row>
     <row r="45" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="139" t="s">
+      <c r="A46" s="142" t="s">
         <v>131</v>
       </c>
-      <c r="B46" s="139"/>
-      <c r="C46" s="139"/>
-      <c r="D46" s="139"/>
-      <c r="E46" s="139"/>
-      <c r="F46" s="139"/>
-      <c r="G46" s="139"/>
-      <c r="H46" s="139"/>
-      <c r="I46" s="139"/>
-      <c r="J46" s="139"/>
-      <c r="K46" s="139"/>
+      <c r="B46" s="142"/>
+      <c r="C46" s="142"/>
+      <c r="D46" s="142"/>
+      <c r="E46" s="142"/>
+      <c r="F46" s="142"/>
+      <c r="G46" s="142"/>
+      <c r="H46" s="142"/>
+      <c r="I46" s="142"/>
+      <c r="J46" s="142"/>
+      <c r="K46" s="142"/>
     </row>
     <row r="47" spans="1:11" s="62" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="60" t="s">
         <v>132</v>
       </c>
       <c r="B47" s="61"/>
-      <c r="C47" s="140" t="s">
+      <c r="C47" s="143" t="s">
         <v>133</v>
       </c>
-      <c r="D47" s="140"/>
-      <c r="E47" s="140"/>
-      <c r="F47" s="140"/>
-      <c r="G47" s="140"/>
-      <c r="H47" s="140"/>
-      <c r="I47" s="140"/>
-      <c r="J47" s="140"/>
-      <c r="K47" s="140"/>
+      <c r="D47" s="143"/>
+      <c r="E47" s="143"/>
+      <c r="F47" s="143"/>
+      <c r="G47" s="143"/>
+      <c r="H47" s="143"/>
+      <c r="I47" s="143"/>
+      <c r="J47" s="143"/>
+      <c r="K47" s="143"/>
     </row>
     <row r="48" spans="1:11" s="64" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="141"/>
-      <c r="B48" s="142" t="s">
+      <c r="A48" s="144"/>
+      <c r="B48" s="145" t="s">
         <v>134</v>
       </c>
-      <c r="C48" s="142" t="s">
+      <c r="C48" s="145" t="s">
         <v>135</v>
       </c>
-      <c r="D48" s="142" t="s">
+      <c r="D48" s="145" t="s">
         <v>136</v>
       </c>
-      <c r="E48" s="142" t="s">
+      <c r="E48" s="145" t="s">
         <v>105</v>
       </c>
-      <c r="F48" s="142" t="s">
+      <c r="F48" s="145" t="s">
         <v>137</v>
       </c>
-      <c r="G48" s="142" t="s">
+      <c r="G48" s="145" t="s">
         <v>109</v>
       </c>
-      <c r="H48" s="143" t="s">
+      <c r="H48" s="146" t="s">
         <v>138</v>
       </c>
-      <c r="I48" s="143"/>
-      <c r="J48" s="143"/>
-      <c r="K48" s="143"/>
+      <c r="I48" s="146"/>
+      <c r="J48" s="146"/>
+      <c r="K48" s="146"/>
     </row>
     <row r="49" spans="1:11" s="64" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="141"/>
-      <c r="B49" s="142"/>
-      <c r="C49" s="142"/>
-      <c r="D49" s="142"/>
-      <c r="E49" s="142"/>
-      <c r="F49" s="142"/>
-      <c r="G49" s="142"/>
-      <c r="H49" s="142" t="s">
+      <c r="A49" s="144"/>
+      <c r="B49" s="145"/>
+      <c r="C49" s="145"/>
+      <c r="D49" s="145"/>
+      <c r="E49" s="145"/>
+      <c r="F49" s="145"/>
+      <c r="G49" s="145"/>
+      <c r="H49" s="145" t="s">
         <v>139</v>
       </c>
-      <c r="I49" s="142"/>
+      <c r="I49" s="145"/>
       <c r="J49" s="63" t="s">
         <v>140</v>
       </c>
@@ -10721,10 +10721,10 @@
       <c r="G50" s="67" t="s">
         <v>110</v>
       </c>
-      <c r="H50" s="146" t="s">
+      <c r="H50" s="150" t="s">
         <v>248</v>
       </c>
-      <c r="I50" s="146"/>
+      <c r="I50" s="150"/>
       <c r="J50" s="67" t="s">
         <v>247</v>
       </c>
@@ -10755,10 +10755,10 @@
       <c r="G51" s="67" t="s">
         <v>110</v>
       </c>
-      <c r="H51" s="144" t="s">
+      <c r="H51" s="149" t="s">
         <v>248</v>
       </c>
-      <c r="I51" s="145"/>
+      <c r="I51" s="148"/>
       <c r="J51" s="67" t="s">
         <v>251</v>
       </c>
@@ -10789,10 +10789,10 @@
       <c r="G52" s="67" t="s">
         <v>110</v>
       </c>
-      <c r="H52" s="144" t="s">
+      <c r="H52" s="149" t="s">
         <v>248</v>
       </c>
-      <c r="I52" s="145"/>
+      <c r="I52" s="148"/>
       <c r="J52" s="67" t="s">
         <v>254</v>
       </c>
@@ -10823,10 +10823,10 @@
       <c r="G53" s="67" t="s">
         <v>110</v>
       </c>
-      <c r="H53" s="144" t="s">
+      <c r="H53" s="149" t="s">
         <v>257</v>
       </c>
-      <c r="I53" s="145"/>
+      <c r="I53" s="148"/>
       <c r="J53" s="67" t="s">
         <v>258</v>
       </c>
@@ -10838,33 +10838,33 @@
       <c r="A54" s="65">
         <v>5</v>
       </c>
-      <c r="B54" s="158" t="s">
+      <c r="B54" s="120" t="s">
         <v>276</v>
       </c>
       <c r="C54" s="66">
         <v>46259</v>
       </c>
-      <c r="D54" s="159" t="s">
+      <c r="D54" s="121" t="s">
         <v>103</v>
       </c>
-      <c r="E54" s="159" t="s">
+      <c r="E54" s="121" t="s">
         <v>108</v>
       </c>
       <c r="F54" s="68" t="str">
         <f t="shared" si="0"/>
         <v>Alta</v>
       </c>
-      <c r="G54" s="159" t="s">
+      <c r="G54" s="121" t="s">
         <v>110</v>
       </c>
-      <c r="H54" s="160" t="s">
+      <c r="H54" s="147" t="s">
         <v>117</v>
       </c>
-      <c r="I54" s="145"/>
-      <c r="J54" s="159" t="s">
+      <c r="I54" s="148"/>
+      <c r="J54" s="121" t="s">
         <v>277</v>
       </c>
-      <c r="K54" s="159" t="s">
+      <c r="K54" s="121" t="s">
         <v>278</v>
       </c>
     </row>
@@ -10872,33 +10872,33 @@
       <c r="A55" s="65">
         <v>6</v>
       </c>
-      <c r="B55" s="158" t="s">
+      <c r="B55" s="120" t="s">
         <v>279</v>
       </c>
       <c r="C55" s="66">
         <v>46259</v>
       </c>
-      <c r="D55" s="159" t="s">
+      <c r="D55" s="121" t="s">
         <v>103</v>
       </c>
-      <c r="E55" s="159" t="s">
+      <c r="E55" s="121" t="s">
         <v>108</v>
       </c>
       <c r="F55" s="68" t="str">
         <f t="shared" si="0"/>
         <v>Alta</v>
       </c>
-      <c r="G55" s="159" t="s">
+      <c r="G55" s="121" t="s">
         <v>110</v>
       </c>
-      <c r="H55" s="160" t="s">
+      <c r="H55" s="147" t="s">
         <v>117</v>
       </c>
-      <c r="I55" s="145"/>
-      <c r="J55" s="159" t="s">
+      <c r="I55" s="148"/>
+      <c r="J55" s="121" t="s">
         <v>280</v>
       </c>
-      <c r="K55" s="159" t="s">
+      <c r="K55" s="121" t="s">
         <v>281</v>
       </c>
     </row>
@@ -10984,116 +10984,116 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" s="53" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="149" t="s">
+      <c r="A1" s="153" t="s">
         <v>143</v>
       </c>
-      <c r="B1" s="149"/>
-      <c r="C1" s="149"/>
-      <c r="D1" s="149"/>
-      <c r="E1" s="149"/>
-      <c r="F1" s="149"/>
-      <c r="G1" s="149"/>
-      <c r="H1" s="149"/>
-      <c r="I1" s="149"/>
-      <c r="J1" s="149"/>
-      <c r="K1" s="149"/>
-      <c r="L1" s="149"/>
-      <c r="M1" s="149"/>
-      <c r="N1" s="149"/>
+      <c r="B1" s="153"/>
+      <c r="C1" s="153"/>
+      <c r="D1" s="153"/>
+      <c r="E1" s="153"/>
+      <c r="F1" s="153"/>
+      <c r="G1" s="153"/>
+      <c r="H1" s="153"/>
+      <c r="I1" s="153"/>
+      <c r="J1" s="153"/>
+      <c r="K1" s="153"/>
+      <c r="L1" s="153"/>
+      <c r="M1" s="153"/>
+      <c r="N1" s="153"/>
     </row>
     <row r="2" spans="1:23" s="69" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="150" t="s">
+      <c r="A2" s="154" t="s">
         <v>127</v>
       </c>
-      <c r="B2" s="150"/>
-      <c r="C2" s="150"/>
-      <c r="D2" s="150"/>
-      <c r="E2" s="150"/>
-      <c r="F2" s="150"/>
-      <c r="G2" s="150"/>
-      <c r="H2" s="150"/>
-      <c r="I2" s="150"/>
-      <c r="J2" s="150"/>
-      <c r="K2" s="150"/>
-      <c r="L2" s="150"/>
-      <c r="M2" s="150"/>
-      <c r="N2" s="150"/>
+      <c r="B2" s="154"/>
+      <c r="C2" s="154"/>
+      <c r="D2" s="154"/>
+      <c r="E2" s="154"/>
+      <c r="F2" s="154"/>
+      <c r="G2" s="154"/>
+      <c r="H2" s="154"/>
+      <c r="I2" s="154"/>
+      <c r="J2" s="154"/>
+      <c r="K2" s="154"/>
+      <c r="L2" s="154"/>
+      <c r="M2" s="154"/>
+      <c r="N2" s="154"/>
     </row>
     <row r="3" spans="1:23" s="69" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="151" t="s">
+      <c r="A3" s="155" t="s">
         <v>144</v>
       </c>
-      <c r="B3" s="151"/>
-      <c r="C3" s="151"/>
-      <c r="D3" s="151"/>
-      <c r="E3" s="151"/>
-      <c r="F3" s="151"/>
-      <c r="G3" s="151"/>
-      <c r="H3" s="151"/>
-      <c r="I3" s="151"/>
-      <c r="J3" s="151"/>
-      <c r="K3" s="151"/>
-      <c r="L3" s="151"/>
-      <c r="M3" s="151"/>
-      <c r="N3" s="151"/>
+      <c r="B3" s="155"/>
+      <c r="C3" s="155"/>
+      <c r="D3" s="155"/>
+      <c r="E3" s="155"/>
+      <c r="F3" s="155"/>
+      <c r="G3" s="155"/>
+      <c r="H3" s="155"/>
+      <c r="I3" s="155"/>
+      <c r="J3" s="155"/>
+      <c r="K3" s="155"/>
+      <c r="L3" s="155"/>
+      <c r="M3" s="155"/>
+      <c r="N3" s="155"/>
     </row>
     <row r="4" spans="1:23" s="69" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="152" t="s">
+      <c r="A4" s="156" t="s">
         <v>145</v>
       </c>
-      <c r="B4" s="152"/>
-      <c r="C4" s="152"/>
-      <c r="D4" s="152"/>
-      <c r="E4" s="152"/>
-      <c r="F4" s="152"/>
-      <c r="G4" s="152"/>
-      <c r="H4" s="152"/>
-      <c r="I4" s="152"/>
-      <c r="J4" s="152"/>
-      <c r="K4" s="152"/>
-      <c r="L4" s="152"/>
-      <c r="M4" s="152"/>
-      <c r="N4" s="152"/>
+      <c r="B4" s="156"/>
+      <c r="C4" s="156"/>
+      <c r="D4" s="156"/>
+      <c r="E4" s="156"/>
+      <c r="F4" s="156"/>
+      <c r="G4" s="156"/>
+      <c r="H4" s="156"/>
+      <c r="I4" s="156"/>
+      <c r="J4" s="156"/>
+      <c r="K4" s="156"/>
+      <c r="L4" s="156"/>
+      <c r="M4" s="156"/>
+      <c r="N4" s="156"/>
     </row>
     <row r="5" spans="1:23" s="69" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="153" t="s">
+      <c r="A5" s="157" t="s">
         <v>146</v>
       </c>
-      <c r="B5" s="153"/>
-      <c r="C5" s="153"/>
-      <c r="D5" s="153"/>
-      <c r="E5" s="153"/>
-      <c r="F5" s="153"/>
-      <c r="G5" s="153"/>
-      <c r="H5" s="153"/>
-      <c r="I5" s="153"/>
-      <c r="J5" s="153"/>
-      <c r="K5" s="153"/>
-      <c r="L5" s="153"/>
-      <c r="M5" s="153"/>
-      <c r="N5" s="153"/>
+      <c r="B5" s="157"/>
+      <c r="C5" s="157"/>
+      <c r="D5" s="157"/>
+      <c r="E5" s="157"/>
+      <c r="F5" s="157"/>
+      <c r="G5" s="157"/>
+      <c r="H5" s="157"/>
+      <c r="I5" s="157"/>
+      <c r="J5" s="157"/>
+      <c r="K5" s="157"/>
+      <c r="L5" s="157"/>
+      <c r="M5" s="157"/>
+      <c r="N5" s="157"/>
     </row>
     <row r="6" spans="1:23" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:23" s="4" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="147" t="s">
+      <c r="A7" s="151" t="s">
         <v>147</v>
       </c>
-      <c r="B7" s="147"/>
-      <c r="D7" s="147" t="s">
+      <c r="B7" s="151"/>
+      <c r="D7" s="151" t="s">
         <v>148</v>
       </c>
-      <c r="E7" s="147"/>
-      <c r="G7" s="147" t="s">
+      <c r="E7" s="151"/>
+      <c r="G7" s="151" t="s">
         <v>149</v>
       </c>
-      <c r="H7" s="147"/>
-      <c r="I7" s="147"/>
-      <c r="J7" s="147"/>
-      <c r="K7" s="147"/>
-      <c r="M7" s="147" t="s">
+      <c r="H7" s="151"/>
+      <c r="I7" s="151"/>
+      <c r="J7" s="151"/>
+      <c r="K7" s="151"/>
+      <c r="M7" s="151" t="s">
         <v>150</v>
       </c>
-      <c r="N7" s="147"/>
+      <c r="N7" s="151"/>
     </row>
     <row r="8" spans="1:23" s="4" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="72" t="s">
@@ -11193,13 +11193,13 @@
       <c r="B11" s="71"/>
       <c r="D11" s="70"/>
       <c r="E11" s="71"/>
-      <c r="G11" s="147" t="s">
+      <c r="G11" s="151" t="s">
         <v>167</v>
       </c>
-      <c r="H11" s="147"/>
-      <c r="I11" s="147"/>
-      <c r="J11" s="147"/>
-      <c r="K11" s="147"/>
+      <c r="H11" s="151"/>
+      <c r="I11" s="151"/>
+      <c r="J11" s="151"/>
+      <c r="K11" s="151"/>
       <c r="M11" s="74" t="s">
         <v>168</v>
       </c>
@@ -11302,12 +11302,12 @@
       <c r="B16" s="71"/>
       <c r="D16" s="70"/>
       <c r="E16" s="71"/>
-      <c r="G16" s="148" t="s">
+      <c r="G16" s="152" t="s">
         <v>177</v>
       </c>
-      <c r="H16" s="148"/>
-      <c r="I16" s="148"/>
-      <c r="J16" s="148"/>
+      <c r="H16" s="152"/>
+      <c r="I16" s="152"/>
+      <c r="J16" s="152"/>
       <c r="K16" s="76">
         <f>SUM(K9,K10,K13,K14,K15)</f>
         <v>14</v>
@@ -11467,42 +11467,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="149" t="s">
+      <c r="A1" s="153" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="149"/>
-      <c r="C1" s="149"/>
-      <c r="D1" s="149"/>
-      <c r="E1" s="149"/>
-      <c r="F1" s="149"/>
-      <c r="G1" s="149"/>
-      <c r="H1" s="149"/>
-      <c r="I1" s="149"/>
-      <c r="J1" s="149"/>
-      <c r="K1" s="149"/>
-      <c r="L1" s="149"/>
-      <c r="M1" s="149"/>
-      <c r="N1" s="149"/>
+      <c r="B1" s="153"/>
+      <c r="C1" s="153"/>
+      <c r="D1" s="153"/>
+      <c r="E1" s="153"/>
+      <c r="F1" s="153"/>
+      <c r="G1" s="153"/>
+      <c r="H1" s="153"/>
+      <c r="I1" s="153"/>
+      <c r="J1" s="153"/>
+      <c r="K1" s="153"/>
+      <c r="L1" s="153"/>
+      <c r="M1" s="153"/>
+      <c r="N1" s="153"/>
     </row>
     <row r="2" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="155" t="s">
+      <c r="A3" s="159" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="155"/>
-      <c r="C3" s="155"/>
-      <c r="E3" s="155" t="s">
+      <c r="B3" s="159"/>
+      <c r="C3" s="159"/>
+      <c r="E3" s="159" t="s">
         <v>190</v>
       </c>
-      <c r="F3" s="155"/>
-      <c r="G3" s="155"/>
-      <c r="H3" s="155"/>
-      <c r="I3" s="155"/>
-      <c r="J3" s="155"/>
-      <c r="K3" s="155"/>
-      <c r="L3" s="155"/>
-      <c r="M3" s="155"/>
-      <c r="N3" s="155"/>
+      <c r="F3" s="159"/>
+      <c r="G3" s="159"/>
+      <c r="H3" s="159"/>
+      <c r="I3" s="159"/>
+      <c r="J3" s="159"/>
+      <c r="K3" s="159"/>
+      <c r="L3" s="159"/>
+      <c r="M3" s="159"/>
+      <c r="N3" s="159"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="83" t="s">
@@ -11515,25 +11515,25 @@
       <c r="C4" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="E4" s="156" t="s">
+      <c r="E4" s="160" t="s">
         <v>192</v>
       </c>
-      <c r="F4" s="154" t="s">
+      <c r="F4" s="158" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="154"/>
-      <c r="H4" s="154" t="s">
+      <c r="G4" s="158"/>
+      <c r="H4" s="158" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="154"/>
-      <c r="J4" s="154" t="s">
+      <c r="I4" s="158"/>
+      <c r="J4" s="158" t="s">
         <v>39</v>
       </c>
-      <c r="K4" s="154"/>
-      <c r="L4" s="154" t="s">
+      <c r="K4" s="158"/>
+      <c r="L4" s="158" t="s">
         <v>40</v>
       </c>
-      <c r="M4" s="154"/>
+      <c r="M4" s="158"/>
       <c r="N4" s="85"/>
     </row>
     <row r="5" spans="1:14" ht="18" x14ac:dyDescent="0.35">
@@ -11546,23 +11546,23 @@
       <c r="C5" s="35" t="s">
         <v>193</v>
       </c>
-      <c r="E5" s="156"/>
-      <c r="F5" s="154" t="s">
+      <c r="E5" s="160"/>
+      <c r="F5" s="158" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="154"/>
-      <c r="H5" s="154" t="s">
+      <c r="G5" s="158"/>
+      <c r="H5" s="158" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="154"/>
-      <c r="J5" s="154" t="s">
+      <c r="I5" s="158"/>
+      <c r="J5" s="158" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="154"/>
-      <c r="L5" s="154" t="s">
+      <c r="K5" s="158"/>
+      <c r="L5" s="158" t="s">
         <v>17</v>
       </c>
-      <c r="M5" s="154"/>
+      <c r="M5" s="158"/>
       <c r="N5" s="38" t="s">
         <v>194</v>
       </c>
@@ -11578,7 +11578,7 @@
       <c r="C6" s="35" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="156"/>
+      <c r="E6" s="160"/>
       <c r="F6" s="88">
         <f>B6*G6</f>
         <v>8.6450000000000014</v>
@@ -12010,11 +12010,11 @@
       <c r="N15" s="95"/>
     </row>
     <row r="16" spans="1:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="A16" s="155" t="s">
+      <c r="A16" s="159" t="s">
         <v>65</v>
       </c>
-      <c r="B16" s="155"/>
-      <c r="C16" s="155"/>
+      <c r="B16" s="159"/>
+      <c r="C16" s="159"/>
       <c r="E16" s="38" t="s">
         <v>214</v>
       </c>

</xml_diff>